<commit_message>
fix(sprint3): align Bug ID / issue column with actual issue numbers
</commit_message>
<xml_diff>
--- a/sprint3/test-cases.xlsx
+++ b/sprint3/test-cases.xlsx
@@ -2574,7 +2574,7 @@
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>BUG-008 (#30)</t>
+          <t>BUG-008 (#31)</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>BUG-009 (#31)</t>
+          <t>BUG-009 (#32)</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
-          <t>BUG-010 (#32)</t>
+          <t>BUG-010 (#33)</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="M52" s="4" t="inlineStr">
         <is>
-          <t>BUG-011 (#33)</t>
+          <t>BUG-011 (#34)</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4468,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>BUG-012 (#34)</t>
+          <t>BUG-012 (#35)</t>
         </is>
       </c>
     </row>

</xml_diff>